<commit_message>
Fix: Hop-rij in het sjabloon stond nog op 8pt zonder tekstterugloop
De eerdere font-/wrap-fix zat alleen in losse preview-bestanden tijdens het
ontwerpen, maar was nooit doorgevoerd in het daadwerkelijke sjabloon dat de
generator gebruikt (Product_Sheet_sjabloon.xlsx) -- dat stond nog op de
originele Blanco-instelling (Hop-kolom Ingredient 8pt, geen wrap, standaard
rijhoogte). Nu gefixt: Hop- en Malt-rij (Ingredient/Name on the label/Order
by size) op 11pt zoals de rest, tekstterugloop aan, rijhoogte naar 45 zodat
de vaak langere teksten (alle hopvarianten, samengevoegde malt+unmalted)
niet worden afgekapt.
</commit_message>
<xml_diff>
--- a/productsheet-generator/Product_Sheet_sjabloon.xlsx
+++ b/productsheet-generator/Product_Sheet_sjabloon.xlsx
@@ -344,7 +344,7 @@
     <numFmt numFmtId="168" formatCode="@"/>
     <numFmt numFmtId="169" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,14 +378,6 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="8"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -729,7 +721,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -753,17 +745,13 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="124">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -775,11 +763,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,11 +775,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -799,7 +787,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -811,7 +799,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -823,7 +811,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -851,28 +839,32 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -887,119 +879,119 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="6" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1007,11 +999,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1023,7 +1015,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1031,7 +1023,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1039,15 +1031,15 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1055,7 +1047,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="21" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="21" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1067,7 +1059,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1075,15 +1067,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1107,7 +1099,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1167,7 +1159,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="25" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="25" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1179,11 +1171,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="27" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="27" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1191,11 +1183,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1208,6 +1200,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1223,7 +1219,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1235,7 +1231,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1243,19 +1239,18 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -1542,7 +1537,7 @@
       <c r="W2" s="4"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -1559,7 +1554,7 @@
       <c r="P3" s="7"/>
       <c r="X3" s="8"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
         <v>1</v>
       </c>
@@ -1578,7 +1573,7 @@
       <c r="P4" s="7"/>
       <c r="X4" s="8"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
         <v>2</v>
       </c>
@@ -1597,7 +1592,7 @@
       <c r="P5" s="7"/>
       <c r="X5" s="8"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
       <c r="D6" s="13"/>
@@ -1614,7 +1609,7 @@
       <c r="P6" s="7"/>
       <c r="X6" s="8"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="16"/>
@@ -1631,7 +1626,7 @@
       <c r="P7" s="7"/>
       <c r="X7" s="8"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="17" t="s">
         <v>3</v>
       </c>
@@ -1675,7 +1670,7 @@
       <c r="P9" s="7"/>
       <c r="X9" s="8"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
         <v>8</v>
       </c>
@@ -1698,29 +1693,29 @@
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
       <c r="D11" s="27"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
-      <c r="N11" s="25"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="29"/>
       <c r="P11" s="7"/>
       <c r="X11" s="8"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="26" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="27"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
       <c r="I12" s="24"/>
       <c r="J12" s="24"/>
       <c r="K12" s="24"/>
@@ -1736,16 +1731,16 @@
       </c>
       <c r="C13" s="26"/>
       <c r="D13" s="27"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29"/>
-      <c r="K13" s="29"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-      <c r="N13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="30"/>
+      <c r="M13" s="30"/>
+      <c r="N13" s="31"/>
       <c r="P13" s="7"/>
       <c r="X13" s="8"/>
     </row>
@@ -1755,50 +1750,50 @@
       </c>
       <c r="C14" s="26"/>
       <c r="D14" s="27"/>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24" t="s">
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="24"/>
-      <c r="N14" s="25"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="28"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="N14" s="29"/>
       <c r="P14" s="7"/>
       <c r="X14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="31"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="24"/>
-      <c r="M15" s="24"/>
-      <c r="N15" s="25"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="28"/>
+      <c r="M15" s="28"/>
+      <c r="N15" s="29"/>
       <c r="P15" s="7"/>
       <c r="X15" s="8"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P16" s="7"/>
-      <c r="Q16" s="33" t="s">
+      <c r="Q16" s="34" t="s">
         <v>15</v>
       </c>
       <c r="X16" s="8"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="17" t="s">
         <v>16</v>
       </c>
@@ -1815,355 +1810,355 @@
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
       <c r="P17" s="7"/>
-      <c r="Q17" s="33" t="s">
+      <c r="Q17" s="34" t="s">
         <v>17</v>
       </c>
       <c r="X17" s="8"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="34" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="35" t="s">
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="35" t="s">
+      <c r="F18" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="36" t="s">
+      <c r="G18" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="H18" s="34" t="s">
+      <c r="H18" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="34"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="35" t="s">
+      <c r="I18" s="35"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="35" t="s">
+      <c r="M18" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="N18" s="35" t="s">
+      <c r="N18" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="33" t="s">
+      <c r="P18" s="38"/>
+      <c r="Q18" s="34" t="s">
         <v>22</v>
       </c>
       <c r="X18" s="8"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="38" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39" t="s">
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="F19" s="40" t="n">
+      <c r="F19" s="41" t="n">
         <v>0.2</v>
       </c>
-      <c r="G19" s="41"/>
-      <c r="H19" s="38" t="s">
+      <c r="G19" s="42"/>
+      <c r="H19" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="I19" s="38"/>
-      <c r="J19" s="38"/>
-      <c r="K19" s="38"/>
-      <c r="L19" s="39" t="s">
+      <c r="I19" s="39"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="M19" s="42" t="s">
+      <c r="M19" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="N19" s="43"/>
+      <c r="N19" s="44"/>
       <c r="P19" s="7"/>
-      <c r="Q19" s="33" t="s">
+      <c r="Q19" s="34" t="s">
         <v>28</v>
       </c>
       <c r="X19" s="8"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="44" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="45" t="s">
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="40" t="n">
+      <c r="F20" s="41" t="n">
         <v>0.3</v>
       </c>
-      <c r="G20" s="46"/>
-      <c r="H20" s="44" t="s">
+      <c r="G20" s="47"/>
+      <c r="H20" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="45" t="s">
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="45"/>
+      <c r="L20" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="M20" s="40" t="n">
+      <c r="M20" s="41" t="n">
         <v>0.1</v>
       </c>
-      <c r="N20" s="46"/>
+      <c r="N20" s="47"/>
       <c r="P20" s="7"/>
-      <c r="Q20" s="33" t="s">
+      <c r="Q20" s="34" t="s">
         <v>32</v>
       </c>
       <c r="X20" s="8"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="44" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="45" t="s">
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="40" t="n">
+      <c r="F21" s="41" t="n">
         <v>0.5</v>
       </c>
-      <c r="G21" s="46"/>
-      <c r="H21" s="44" t="s">
+      <c r="G21" s="47"/>
+      <c r="H21" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44"/>
-      <c r="K21" s="44"/>
-      <c r="L21" s="45" t="s">
+      <c r="I21" s="45"/>
+      <c r="J21" s="45"/>
+      <c r="K21" s="45"/>
+      <c r="L21" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="M21" s="40" t="n">
+      <c r="M21" s="41" t="n">
         <v>0.1</v>
       </c>
-      <c r="N21" s="46"/>
+      <c r="N21" s="47"/>
       <c r="P21" s="7"/>
-      <c r="Q21" s="33" t="s">
+      <c r="Q21" s="34" t="s">
         <v>36</v>
       </c>
       <c r="X21" s="8"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="44" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45" t="s">
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="42" t="n">
+      <c r="F22" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="47"/>
-      <c r="H22" s="44" t="s">
+      <c r="G22" s="48"/>
+      <c r="H22" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44"/>
-      <c r="K22" s="44"/>
-      <c r="L22" s="45" t="s">
+      <c r="I22" s="45"/>
+      <c r="J22" s="45"/>
+      <c r="K22" s="45"/>
+      <c r="L22" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="M22" s="40" t="n">
+      <c r="M22" s="41" t="n">
         <v>0.1</v>
       </c>
-      <c r="N22" s="47"/>
+      <c r="N22" s="48"/>
       <c r="P22" s="7"/>
-      <c r="Q22" s="33" t="s">
+      <c r="Q22" s="34" t="s">
         <v>41</v>
       </c>
       <c r="X22" s="8"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="44" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45" t="s">
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="42" t="n">
+      <c r="F23" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="G23" s="47"/>
-      <c r="H23" s="44" t="s">
+      <c r="G23" s="48"/>
+      <c r="H23" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44"/>
-      <c r="K23" s="44"/>
-      <c r="L23" s="45" t="s">
+      <c r="I23" s="45"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="45"/>
+      <c r="L23" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="M23" s="40" t="s">
+      <c r="M23" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="N23" s="47"/>
+      <c r="N23" s="48"/>
       <c r="P23" s="7"/>
-      <c r="Q23" s="33" t="s">
+      <c r="Q23" s="34" t="s">
         <v>44</v>
       </c>
       <c r="X23" s="8"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="44" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="40" t="n">
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="41" t="n">
         <v>0.2</v>
       </c>
-      <c r="G24" s="46"/>
-      <c r="H24" s="48" t="s">
+      <c r="G24" s="47"/>
+      <c r="H24" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="I24" s="48"/>
-      <c r="J24" s="48"/>
-      <c r="K24" s="48"/>
-      <c r="L24" s="45" t="s">
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="M24" s="40" t="s">
+      <c r="M24" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="49" t="n">
+      <c r="N24" s="50" t="n">
         <v>50</v>
       </c>
       <c r="P24" s="7"/>
       <c r="X24" s="8"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="50" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="51"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="53" t="s">
+      <c r="C25" s="52"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="F25" s="54" t="s">
+      <c r="F25" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="G25" s="55"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="51"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="52"/>
-      <c r="L25" s="53"/>
-      <c r="M25" s="56"/>
-      <c r="N25" s="55"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="52"/>
+      <c r="J25" s="52"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="54"/>
+      <c r="M25" s="57"/>
+      <c r="N25" s="56"/>
       <c r="P25" s="7"/>
       <c r="X25" s="8"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P26" s="7"/>
       <c r="X26" s="8"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="18" t="s">
         <v>48</v>
       </c>
       <c r="C27" s="18"/>
       <c r="D27" s="23"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="57"/>
-      <c r="L27" s="57"/>
-      <c r="M27" s="57"/>
-      <c r="N27" s="57"/>
+      <c r="E27" s="58"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="58"/>
+      <c r="J27" s="58"/>
+      <c r="K27" s="58"/>
+      <c r="L27" s="58"/>
+      <c r="M27" s="58"/>
+      <c r="N27" s="58"/>
       <c r="P27" s="7"/>
       <c r="X27" s="8"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="58"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="59"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="57"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="57"/>
-      <c r="K28" s="57"/>
-      <c r="L28" s="57"/>
-      <c r="M28" s="57"/>
-      <c r="N28" s="57"/>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="59"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="60"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58"/>
+      <c r="H28" s="58"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="58"/>
+      <c r="K28" s="58"/>
+      <c r="L28" s="58"/>
+      <c r="M28" s="58"/>
+      <c r="N28" s="58"/>
       <c r="P28" s="7"/>
       <c r="X28" s="8"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="58"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="57"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="57"/>
-      <c r="H29" s="57"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="57"/>
-      <c r="K29" s="57"/>
-      <c r="L29" s="57"/>
-      <c r="M29" s="57"/>
-      <c r="N29" s="57"/>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="59"/>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58"/>
+      <c r="K29" s="58"/>
+      <c r="L29" s="58"/>
+      <c r="M29" s="58"/>
+      <c r="N29" s="58"/>
       <c r="P29" s="7"/>
       <c r="X29" s="8"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="58"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="57"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="57"/>
-      <c r="H30" s="57"/>
-      <c r="I30" s="57"/>
-      <c r="J30" s="57"/>
-      <c r="K30" s="57"/>
-      <c r="L30" s="57"/>
-      <c r="M30" s="57"/>
-      <c r="N30" s="57"/>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="59"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="58"/>
+      <c r="F30" s="58"/>
+      <c r="G30" s="58"/>
+      <c r="H30" s="58"/>
+      <c r="I30" s="58"/>
+      <c r="J30" s="58"/>
+      <c r="K30" s="58"/>
+      <c r="L30" s="58"/>
+      <c r="M30" s="58"/>
+      <c r="N30" s="58"/>
       <c r="P30" s="7"/>
       <c r="X30" s="8"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="60"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="57"/>
-      <c r="F31" s="57"/>
-      <c r="G31" s="57"/>
-      <c r="H31" s="57"/>
-      <c r="I31" s="57"/>
-      <c r="J31" s="57"/>
-      <c r="K31" s="57"/>
-      <c r="L31" s="57"/>
-      <c r="M31" s="57"/>
-      <c r="N31" s="57"/>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="61"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
+      <c r="G31" s="58"/>
+      <c r="H31" s="58"/>
+      <c r="I31" s="58"/>
+      <c r="J31" s="58"/>
+      <c r="K31" s="58"/>
+      <c r="L31" s="58"/>
+      <c r="M31" s="58"/>
+      <c r="N31" s="58"/>
       <c r="P31" s="7"/>
       <c r="X31" s="8"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P32" s="7"/>
       <c r="X32" s="8"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="17" t="s">
         <v>49</v>
       </c>
@@ -2182,282 +2177,282 @@
       <c r="P33" s="7"/>
       <c r="X33" s="8"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="22" t="s">
         <v>50</v>
       </c>
       <c r="C34" s="22"/>
-      <c r="D34" s="59"/>
-      <c r="E34" s="61" t="n">
+      <c r="D34" s="60"/>
+      <c r="E34" s="62" t="n">
         <f aca="false">G21</f>
         <v>0</v>
       </c>
-      <c r="F34" s="61"/>
-      <c r="G34" s="61"/>
-      <c r="H34" s="61"/>
-      <c r="I34" s="61"/>
-      <c r="J34" s="61"/>
-      <c r="K34" s="61"/>
-      <c r="L34" s="61"/>
-      <c r="M34" s="61"/>
-      <c r="N34" s="61"/>
-      <c r="P34" s="62"/>
-      <c r="Q34" s="63"/>
-      <c r="R34" s="63"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="62"/>
+      <c r="H34" s="62"/>
+      <c r="I34" s="62"/>
+      <c r="J34" s="62"/>
+      <c r="K34" s="62"/>
+      <c r="L34" s="62"/>
+      <c r="M34" s="62"/>
+      <c r="N34" s="62"/>
+      <c r="P34" s="63"/>
+      <c r="Q34" s="64"/>
+      <c r="R34" s="64"/>
       <c r="X34" s="8"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="26" t="s">
         <v>51</v>
       </c>
       <c r="C35" s="26"/>
       <c r="D35" s="27"/>
-      <c r="E35" s="64" t="n">
+      <c r="E35" s="65" t="n">
         <f aca="false">G19</f>
         <v>0</v>
       </c>
-      <c r="F35" s="64"/>
-      <c r="G35" s="64"/>
-      <c r="H35" s="64"/>
-      <c r="I35" s="64"/>
-      <c r="J35" s="64"/>
-      <c r="K35" s="64"/>
-      <c r="L35" s="64"/>
-      <c r="M35" s="64"/>
-      <c r="N35" s="64"/>
-      <c r="P35" s="62"/>
-      <c r="Q35" s="63"/>
-      <c r="R35" s="63"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
+      <c r="K35" s="65"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="65"/>
+      <c r="N35" s="65"/>
+      <c r="P35" s="63"/>
+      <c r="Q35" s="64"/>
+      <c r="R35" s="64"/>
       <c r="X35" s="8"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C36" s="26"/>
       <c r="D36" s="27"/>
-      <c r="E36" s="65" t="n">
+      <c r="E36" s="66" t="n">
         <f aca="false">G23</f>
         <v>0</v>
       </c>
-      <c r="F36" s="65"/>
-      <c r="G36" s="65"/>
-      <c r="H36" s="65"/>
-      <c r="I36" s="65"/>
-      <c r="J36" s="65"/>
-      <c r="K36" s="65"/>
-      <c r="L36" s="65"/>
-      <c r="M36" s="65"/>
-      <c r="N36" s="65"/>
-      <c r="P36" s="62"/>
-      <c r="Q36" s="63"/>
-      <c r="R36" s="63"/>
+      <c r="F36" s="66"/>
+      <c r="G36" s="66"/>
+      <c r="H36" s="66"/>
+      <c r="I36" s="66"/>
+      <c r="J36" s="66"/>
+      <c r="K36" s="66"/>
+      <c r="L36" s="66"/>
+      <c r="M36" s="66"/>
+      <c r="N36" s="66"/>
+      <c r="P36" s="63"/>
+      <c r="Q36" s="64"/>
+      <c r="R36" s="64"/>
       <c r="X36" s="8"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="26" t="s">
         <v>53</v>
       </c>
       <c r="C37" s="26"/>
       <c r="D37" s="27"/>
-      <c r="E37" s="64"/>
-      <c r="F37" s="64"/>
-      <c r="G37" s="64"/>
-      <c r="H37" s="64"/>
-      <c r="I37" s="64"/>
-      <c r="J37" s="64"/>
-      <c r="K37" s="64"/>
-      <c r="L37" s="64"/>
-      <c r="M37" s="64"/>
-      <c r="N37" s="64"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="65"/>
+      <c r="K37" s="65"/>
+      <c r="L37" s="65"/>
+      <c r="M37" s="65"/>
+      <c r="N37" s="65"/>
       <c r="P37" s="7"/>
       <c r="X37" s="8"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="26" t="s">
         <v>54</v>
       </c>
       <c r="C38" s="26"/>
       <c r="D38" s="27"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="65"/>
-      <c r="H38" s="65"/>
-      <c r="I38" s="65"/>
-      <c r="J38" s="65"/>
-      <c r="K38" s="65"/>
-      <c r="L38" s="65"/>
-      <c r="M38" s="65"/>
-      <c r="N38" s="65"/>
+      <c r="E38" s="66"/>
+      <c r="F38" s="66"/>
+      <c r="G38" s="66"/>
+      <c r="H38" s="66"/>
+      <c r="I38" s="66"/>
+      <c r="J38" s="66"/>
+      <c r="K38" s="66"/>
+      <c r="L38" s="66"/>
+      <c r="M38" s="66"/>
+      <c r="N38" s="66"/>
       <c r="P38" s="7"/>
       <c r="X38" s="8"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="26" t="s">
         <v>55</v>
       </c>
       <c r="C39" s="26"/>
       <c r="D39" s="27"/>
-      <c r="E39" s="65" t="n">
+      <c r="E39" s="66" t="n">
         <f aca="false">G22</f>
         <v>0</v>
       </c>
-      <c r="F39" s="65"/>
-      <c r="G39" s="65"/>
-      <c r="H39" s="65"/>
-      <c r="I39" s="65"/>
-      <c r="J39" s="65"/>
-      <c r="K39" s="65"/>
-      <c r="L39" s="65"/>
-      <c r="M39" s="65"/>
-      <c r="N39" s="65"/>
-      <c r="P39" s="62"/>
-      <c r="Q39" s="63"/>
-      <c r="R39" s="63"/>
+      <c r="F39" s="66"/>
+      <c r="G39" s="66"/>
+      <c r="H39" s="66"/>
+      <c r="I39" s="66"/>
+      <c r="J39" s="66"/>
+      <c r="K39" s="66"/>
+      <c r="L39" s="66"/>
+      <c r="M39" s="66"/>
+      <c r="N39" s="66"/>
+      <c r="P39" s="63"/>
+      <c r="Q39" s="64"/>
+      <c r="R39" s="64"/>
       <c r="X39" s="8"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="26" t="s">
         <v>56</v>
       </c>
       <c r="C40" s="26"/>
       <c r="D40" s="27"/>
-      <c r="E40" s="65"/>
-      <c r="F40" s="65"/>
-      <c r="G40" s="65"/>
-      <c r="H40" s="65"/>
-      <c r="I40" s="65"/>
-      <c r="J40" s="65"/>
-      <c r="K40" s="65"/>
-      <c r="L40" s="65"/>
-      <c r="M40" s="65"/>
-      <c r="N40" s="65"/>
-      <c r="P40" s="62"/>
-      <c r="Q40" s="63"/>
-      <c r="R40" s="63"/>
+      <c r="E40" s="66"/>
+      <c r="F40" s="66"/>
+      <c r="G40" s="66"/>
+      <c r="H40" s="66"/>
+      <c r="I40" s="66"/>
+      <c r="J40" s="66"/>
+      <c r="K40" s="66"/>
+      <c r="L40" s="66"/>
+      <c r="M40" s="66"/>
+      <c r="N40" s="66"/>
+      <c r="P40" s="63"/>
+      <c r="Q40" s="64"/>
+      <c r="R40" s="64"/>
       <c r="X40" s="8"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="26" t="s">
         <v>57</v>
       </c>
       <c r="C41" s="26"/>
       <c r="D41" s="27"/>
-      <c r="E41" s="66"/>
-      <c r="F41" s="66"/>
-      <c r="G41" s="66"/>
-      <c r="H41" s="66"/>
-      <c r="I41" s="66"/>
-      <c r="J41" s="66"/>
-      <c r="K41" s="66"/>
-      <c r="L41" s="66"/>
-      <c r="M41" s="66"/>
-      <c r="N41" s="66"/>
+      <c r="E41" s="67"/>
+      <c r="F41" s="67"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="67"/>
+      <c r="I41" s="67"/>
+      <c r="J41" s="67"/>
+      <c r="K41" s="67"/>
+      <c r="L41" s="67"/>
+      <c r="M41" s="67"/>
+      <c r="N41" s="67"/>
       <c r="P41" s="7"/>
       <c r="X41" s="8"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="67" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="C42" s="67"/>
-      <c r="D42" s="68"/>
-      <c r="E42" s="69"/>
-      <c r="F42" s="69"/>
-      <c r="G42" s="69"/>
-      <c r="H42" s="69"/>
-      <c r="I42" s="69"/>
-      <c r="J42" s="69"/>
-      <c r="K42" s="69"/>
-      <c r="L42" s="69"/>
-      <c r="M42" s="69"/>
-      <c r="N42" s="69"/>
-      <c r="P42" s="70" t="s">
+      <c r="C42" s="68"/>
+      <c r="D42" s="69"/>
+      <c r="E42" s="70"/>
+      <c r="F42" s="70"/>
+      <c r="G42" s="70"/>
+      <c r="H42" s="70"/>
+      <c r="I42" s="70"/>
+      <c r="J42" s="70"/>
+      <c r="K42" s="70"/>
+      <c r="L42" s="70"/>
+      <c r="M42" s="70"/>
+      <c r="N42" s="70"/>
+      <c r="P42" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="Q42" s="71"/>
-      <c r="R42" s="71"/>
-      <c r="S42" s="71"/>
-      <c r="T42" s="71"/>
-      <c r="U42" s="71"/>
-      <c r="V42" s="71"/>
-      <c r="W42" s="71"/>
-      <c r="X42" s="72"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P43" s="70" t="s">
+      <c r="Q42" s="72"/>
+      <c r="R42" s="72"/>
+      <c r="S42" s="72"/>
+      <c r="T42" s="72"/>
+      <c r="U42" s="72"/>
+      <c r="V42" s="72"/>
+      <c r="W42" s="72"/>
+      <c r="X42" s="73"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P43" s="71" t="s">
         <v>60</v>
       </c>
-      <c r="Q43" s="71"/>
-      <c r="R43" s="71"/>
-      <c r="S43" s="71"/>
-      <c r="T43" s="71"/>
-      <c r="U43" s="71"/>
-      <c r="V43" s="71"/>
-      <c r="W43" s="71"/>
-      <c r="X43" s="72"/>
+      <c r="Q43" s="72"/>
+      <c r="R43" s="72"/>
+      <c r="S43" s="72"/>
+      <c r="T43" s="72"/>
+      <c r="U43" s="72"/>
+      <c r="V43" s="72"/>
+      <c r="W43" s="72"/>
+      <c r="X43" s="73"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="73" t="s">
+      <c r="B44" s="74" t="s">
         <v>61</v>
       </c>
-      <c r="C44" s="73"/>
-      <c r="D44" s="74"/>
-      <c r="E44" s="75"/>
-      <c r="F44" s="75"/>
-      <c r="G44" s="75"/>
-      <c r="H44" s="76"/>
-      <c r="I44" s="76"/>
-      <c r="J44" s="76"/>
-      <c r="K44" s="76"/>
-      <c r="L44" s="76"/>
-      <c r="M44" s="75"/>
-      <c r="N44" s="75"/>
-      <c r="P44" s="70" t="s">
+      <c r="C44" s="74"/>
+      <c r="D44" s="75"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="77"/>
+      <c r="I44" s="77"/>
+      <c r="J44" s="77"/>
+      <c r="K44" s="77"/>
+      <c r="L44" s="77"/>
+      <c r="M44" s="76"/>
+      <c r="N44" s="76"/>
+      <c r="P44" s="71" t="s">
         <v>62</v>
       </c>
-      <c r="Q44" s="71"/>
-      <c r="R44" s="71"/>
-      <c r="S44" s="71"/>
-      <c r="T44" s="71"/>
-      <c r="U44" s="71"/>
-      <c r="V44" s="71"/>
-      <c r="W44" s="71"/>
-      <c r="X44" s="72"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="73"/>
-      <c r="C45" s="73"/>
-      <c r="D45" s="77"/>
-      <c r="E45" s="78"/>
-      <c r="F45" s="78"/>
-      <c r="G45" s="78"/>
-      <c r="H45" s="75"/>
-      <c r="I45" s="75"/>
-      <c r="J45" s="75"/>
-      <c r="K45" s="75"/>
-      <c r="L45" s="75"/>
-      <c r="M45" s="76"/>
-      <c r="N45" s="76"/>
-      <c r="P45" s="70" t="s">
+      <c r="Q44" s="72"/>
+      <c r="R44" s="72"/>
+      <c r="S44" s="72"/>
+      <c r="T44" s="72"/>
+      <c r="U44" s="72"/>
+      <c r="V44" s="72"/>
+      <c r="W44" s="72"/>
+      <c r="X44" s="73"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="74"/>
+      <c r="C45" s="74"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="79"/>
+      <c r="F45" s="79"/>
+      <c r="G45" s="79"/>
+      <c r="H45" s="76"/>
+      <c r="I45" s="76"/>
+      <c r="J45" s="76"/>
+      <c r="K45" s="76"/>
+      <c r="L45" s="76"/>
+      <c r="M45" s="77"/>
+      <c r="N45" s="77"/>
+      <c r="P45" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="Q45" s="71"/>
-      <c r="R45" s="71"/>
-      <c r="S45" s="71"/>
-      <c r="T45" s="71"/>
-      <c r="U45" s="71"/>
-      <c r="V45" s="71"/>
-      <c r="W45" s="71"/>
-      <c r="X45" s="72"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q45" s="72"/>
+      <c r="R45" s="72"/>
+      <c r="S45" s="72"/>
+      <c r="T45" s="72"/>
+      <c r="U45" s="72"/>
+      <c r="V45" s="72"/>
+      <c r="W45" s="72"/>
+      <c r="X45" s="73"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P46" s="7" t="s">
         <v>64</v>
       </c>
       <c r="X46" s="8"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="17" t="s">
         <v>65</v>
       </c>
@@ -2473,17 +2468,17 @@
       <c r="L47" s="17"/>
       <c r="M47" s="17"/>
       <c r="N47" s="17"/>
-      <c r="P47" s="79" t="s">
+      <c r="P47" s="80" t="s">
         <v>66</v>
       </c>
-      <c r="Q47" s="80"/>
-      <c r="R47" s="80"/>
-      <c r="S47" s="80"/>
-      <c r="T47" s="80"/>
-      <c r="U47" s="80"/>
-      <c r="V47" s="80"/>
-      <c r="W47" s="80"/>
-      <c r="X47" s="81"/>
+      <c r="Q47" s="81"/>
+      <c r="R47" s="81"/>
+      <c r="S47" s="81"/>
+      <c r="T47" s="81"/>
+      <c r="U47" s="81"/>
+      <c r="V47" s="81"/>
+      <c r="W47" s="81"/>
+      <c r="X47" s="82"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="26" t="s">
@@ -2491,18 +2486,18 @@
       </c>
       <c r="C48" s="26"/>
       <c r="D48" s="27"/>
-      <c r="E48" s="65" t="s">
+      <c r="E48" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="F48" s="65"/>
-      <c r="G48" s="65"/>
-      <c r="H48" s="65"/>
-      <c r="I48" s="65"/>
-      <c r="J48" s="65"/>
-      <c r="K48" s="65"/>
-      <c r="L48" s="65"/>
-      <c r="M48" s="65"/>
-      <c r="N48" s="65"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="66"/>
+      <c r="H48" s="66"/>
+      <c r="I48" s="66"/>
+      <c r="J48" s="66"/>
+      <c r="K48" s="66"/>
+      <c r="L48" s="66"/>
+      <c r="M48" s="66"/>
+      <c r="N48" s="66"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="26" t="s">
@@ -2510,116 +2505,116 @@
       </c>
       <c r="C49" s="26"/>
       <c r="D49" s="27"/>
-      <c r="E49" s="65" t="s">
+      <c r="E49" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="F49" s="65"/>
-      <c r="G49" s="65"/>
-      <c r="H49" s="65"/>
-      <c r="I49" s="65"/>
-      <c r="J49" s="65"/>
-      <c r="K49" s="65"/>
-      <c r="L49" s="65"/>
-      <c r="M49" s="65"/>
-      <c r="N49" s="65"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="82" t="s">
+      <c r="F49" s="66"/>
+      <c r="G49" s="66"/>
+      <c r="H49" s="66"/>
+      <c r="I49" s="66"/>
+      <c r="J49" s="66"/>
+      <c r="K49" s="66"/>
+      <c r="L49" s="66"/>
+      <c r="M49" s="66"/>
+      <c r="N49" s="66"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B50" s="83" t="s">
         <v>70</v>
       </c>
-      <c r="C50" s="83"/>
-      <c r="D50" s="68"/>
-      <c r="E50" s="84" t="s">
+      <c r="C50" s="84"/>
+      <c r="D50" s="69"/>
+      <c r="E50" s="85" t="s">
         <v>68</v>
       </c>
-      <c r="F50" s="84"/>
-      <c r="G50" s="84"/>
-      <c r="H50" s="84"/>
-      <c r="I50" s="84"/>
-      <c r="J50" s="84"/>
-      <c r="K50" s="84"/>
-      <c r="L50" s="84"/>
-      <c r="M50" s="84"/>
+      <c r="F50" s="85"/>
+      <c r="G50" s="85"/>
+      <c r="H50" s="85"/>
+      <c r="I50" s="85"/>
+      <c r="J50" s="85"/>
+      <c r="K50" s="85"/>
+      <c r="L50" s="85"/>
+      <c r="M50" s="85"/>
       <c r="N50" s="14"/>
     </row>
     <row r="52" customFormat="false" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="85" t="s">
+      <c r="B52" s="86" t="s">
         <v>71</v>
       </c>
-      <c r="C52" s="86"/>
+      <c r="C52" s="87"/>
       <c r="D52" s="23"/>
-      <c r="E52" s="87"/>
-      <c r="F52" s="87"/>
-      <c r="G52" s="87"/>
-      <c r="H52" s="87"/>
-      <c r="I52" s="87"/>
-      <c r="J52" s="88"/>
-      <c r="K52" s="88"/>
-      <c r="L52" s="88"/>
-      <c r="M52" s="88"/>
-      <c r="N52" s="89"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="90"/>
-      <c r="C53" s="91"/>
-      <c r="D53" s="59"/>
-      <c r="E53" s="92"/>
-      <c r="F53" s="93"/>
-      <c r="G53" s="93"/>
-      <c r="H53" s="93"/>
-      <c r="I53" s="93"/>
-      <c r="J53" s="93"/>
-      <c r="K53" s="93"/>
-      <c r="L53" s="93"/>
-      <c r="M53" s="93"/>
-      <c r="N53" s="94"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="90"/>
-      <c r="C54" s="91"/>
-      <c r="D54" s="59"/>
-      <c r="E54" s="92"/>
-      <c r="F54" s="93"/>
-      <c r="G54" s="93"/>
-      <c r="H54" s="93"/>
-      <c r="I54" s="93"/>
-      <c r="J54" s="93"/>
-      <c r="K54" s="93"/>
-      <c r="L54" s="93"/>
-      <c r="M54" s="93"/>
-      <c r="N54" s="94"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="90"/>
-      <c r="C55" s="91"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="92"/>
-      <c r="F55" s="93"/>
-      <c r="G55" s="93"/>
-      <c r="H55" s="93"/>
-      <c r="I55" s="93"/>
-      <c r="J55" s="93"/>
-      <c r="K55" s="93"/>
-      <c r="L55" s="93"/>
-      <c r="M55" s="93"/>
-      <c r="N55" s="94"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="95"/>
-      <c r="C56" s="96"/>
-      <c r="D56" s="32"/>
-      <c r="E56" s="97"/>
-      <c r="F56" s="98"/>
-      <c r="G56" s="98"/>
-      <c r="H56" s="98"/>
-      <c r="I56" s="98"/>
-      <c r="J56" s="98"/>
-      <c r="K56" s="98"/>
-      <c r="L56" s="98"/>
-      <c r="M56" s="98"/>
-      <c r="N56" s="99"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E52" s="88"/>
+      <c r="F52" s="88"/>
+      <c r="G52" s="88"/>
+      <c r="H52" s="88"/>
+      <c r="I52" s="88"/>
+      <c r="J52" s="89"/>
+      <c r="K52" s="89"/>
+      <c r="L52" s="89"/>
+      <c r="M52" s="89"/>
+      <c r="N52" s="90"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="91"/>
+      <c r="C53" s="92"/>
+      <c r="D53" s="60"/>
+      <c r="E53" s="93"/>
+      <c r="F53" s="94"/>
+      <c r="G53" s="94"/>
+      <c r="H53" s="94"/>
+      <c r="I53" s="94"/>
+      <c r="J53" s="94"/>
+      <c r="K53" s="94"/>
+      <c r="L53" s="94"/>
+      <c r="M53" s="94"/>
+      <c r="N53" s="95"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="91"/>
+      <c r="C54" s="92"/>
+      <c r="D54" s="60"/>
+      <c r="E54" s="93"/>
+      <c r="F54" s="94"/>
+      <c r="G54" s="94"/>
+      <c r="H54" s="94"/>
+      <c r="I54" s="94"/>
+      <c r="J54" s="94"/>
+      <c r="K54" s="94"/>
+      <c r="L54" s="94"/>
+      <c r="M54" s="94"/>
+      <c r="N54" s="95"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="91"/>
+      <c r="C55" s="92"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="93"/>
+      <c r="F55" s="94"/>
+      <c r="G55" s="94"/>
+      <c r="H55" s="94"/>
+      <c r="I55" s="94"/>
+      <c r="J55" s="94"/>
+      <c r="K55" s="94"/>
+      <c r="L55" s="94"/>
+      <c r="M55" s="94"/>
+      <c r="N55" s="95"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="96"/>
+      <c r="C56" s="97"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="98"/>
+      <c r="F56" s="99"/>
+      <c r="G56" s="99"/>
+      <c r="H56" s="99"/>
+      <c r="I56" s="99"/>
+      <c r="J56" s="99"/>
+      <c r="K56" s="99"/>
+      <c r="L56" s="99"/>
+      <c r="M56" s="99"/>
+      <c r="N56" s="100"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="17" t="s">
         <v>72</v>
       </c>
@@ -2636,181 +2631,181 @@
       <c r="M58" s="17"/>
       <c r="N58" s="17"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="26" t="s">
         <v>73</v>
       </c>
       <c r="C59" s="26"/>
       <c r="D59" s="27"/>
-      <c r="E59" s="65"/>
-      <c r="F59" s="65"/>
-      <c r="G59" s="65"/>
-      <c r="H59" s="65"/>
-      <c r="I59" s="65"/>
-      <c r="J59" s="65"/>
-      <c r="K59" s="65"/>
-      <c r="L59" s="65"/>
-      <c r="M59" s="65"/>
-      <c r="N59" s="65"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E59" s="66"/>
+      <c r="F59" s="66"/>
+      <c r="G59" s="66"/>
+      <c r="H59" s="66"/>
+      <c r="I59" s="66"/>
+      <c r="J59" s="66"/>
+      <c r="K59" s="66"/>
+      <c r="L59" s="66"/>
+      <c r="M59" s="66"/>
+      <c r="N59" s="66"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="26" t="s">
         <v>74</v>
       </c>
       <c r="C60" s="26"/>
       <c r="D60" s="27"/>
-      <c r="E60" s="65"/>
-      <c r="F60" s="65"/>
-      <c r="G60" s="65"/>
-      <c r="H60" s="65"/>
-      <c r="I60" s="65"/>
-      <c r="J60" s="65"/>
-      <c r="K60" s="65"/>
-      <c r="L60" s="65"/>
-      <c r="M60" s="65"/>
-      <c r="N60" s="65"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="100" t="s">
+      <c r="E60" s="66"/>
+      <c r="F60" s="66"/>
+      <c r="G60" s="66"/>
+      <c r="H60" s="66"/>
+      <c r="I60" s="66"/>
+      <c r="J60" s="66"/>
+      <c r="K60" s="66"/>
+      <c r="L60" s="66"/>
+      <c r="M60" s="66"/>
+      <c r="N60" s="66"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B61" s="101" t="s">
         <v>75</v>
       </c>
-      <c r="C61" s="101"/>
-      <c r="D61" s="102"/>
-      <c r="E61" s="103"/>
-      <c r="F61" s="103"/>
-      <c r="G61" s="103"/>
-      <c r="H61" s="103"/>
-      <c r="I61" s="103"/>
-      <c r="J61" s="103"/>
-      <c r="K61" s="103"/>
-      <c r="L61" s="103"/>
-      <c r="M61" s="103"/>
-      <c r="N61" s="104"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="100" t="s">
+      <c r="C61" s="102"/>
+      <c r="D61" s="103"/>
+      <c r="E61" s="104"/>
+      <c r="F61" s="104"/>
+      <c r="G61" s="104"/>
+      <c r="H61" s="104"/>
+      <c r="I61" s="104"/>
+      <c r="J61" s="104"/>
+      <c r="K61" s="104"/>
+      <c r="L61" s="104"/>
+      <c r="M61" s="104"/>
+      <c r="N61" s="105"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B62" s="101" t="s">
         <v>76</v>
       </c>
-      <c r="C62" s="101"/>
-      <c r="D62" s="102"/>
-      <c r="E62" s="103"/>
-      <c r="F62" s="103"/>
-      <c r="G62" s="103"/>
-      <c r="H62" s="103"/>
-      <c r="I62" s="103"/>
-      <c r="J62" s="103"/>
-      <c r="K62" s="103"/>
-      <c r="L62" s="103"/>
-      <c r="M62" s="103"/>
-      <c r="N62" s="104"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="100" t="s">
+      <c r="C62" s="102"/>
+      <c r="D62" s="103"/>
+      <c r="E62" s="104"/>
+      <c r="F62" s="104"/>
+      <c r="G62" s="104"/>
+      <c r="H62" s="104"/>
+      <c r="I62" s="104"/>
+      <c r="J62" s="104"/>
+      <c r="K62" s="104"/>
+      <c r="L62" s="104"/>
+      <c r="M62" s="104"/>
+      <c r="N62" s="105"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B63" s="101" t="s">
         <v>77</v>
       </c>
-      <c r="C63" s="101"/>
-      <c r="D63" s="102"/>
-      <c r="E63" s="103"/>
-      <c r="F63" s="103"/>
-      <c r="G63" s="103"/>
-      <c r="H63" s="103"/>
-      <c r="I63" s="103"/>
-      <c r="J63" s="103"/>
-      <c r="K63" s="103"/>
-      <c r="L63" s="103"/>
-      <c r="M63" s="103"/>
-      <c r="N63" s="104"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="82" t="s">
+      <c r="C63" s="102"/>
+      <c r="D63" s="103"/>
+      <c r="E63" s="104"/>
+      <c r="F63" s="104"/>
+      <c r="G63" s="104"/>
+      <c r="H63" s="104"/>
+      <c r="I63" s="104"/>
+      <c r="J63" s="104"/>
+      <c r="K63" s="104"/>
+      <c r="L63" s="104"/>
+      <c r="M63" s="104"/>
+      <c r="N63" s="105"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B64" s="83" t="s">
         <v>78</v>
       </c>
-      <c r="C64" s="83"/>
-      <c r="D64" s="68"/>
-      <c r="E64" s="84"/>
-      <c r="F64" s="84"/>
-      <c r="G64" s="84"/>
-      <c r="H64" s="84"/>
-      <c r="I64" s="84"/>
-      <c r="J64" s="84"/>
-      <c r="K64" s="84"/>
-      <c r="L64" s="84"/>
-      <c r="M64" s="84"/>
+      <c r="C64" s="84"/>
+      <c r="D64" s="69"/>
+      <c r="E64" s="85"/>
+      <c r="F64" s="85"/>
+      <c r="G64" s="85"/>
+      <c r="H64" s="85"/>
+      <c r="I64" s="85"/>
+      <c r="J64" s="85"/>
+      <c r="K64" s="85"/>
+      <c r="L64" s="85"/>
+      <c r="M64" s="85"/>
       <c r="N64" s="14"/>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="105" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B66" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="C66" s="106"/>
-      <c r="D66" s="74"/>
-      <c r="E66" s="107"/>
-      <c r="F66" s="107"/>
-      <c r="G66" s="107"/>
-      <c r="H66" s="107"/>
-      <c r="I66" s="107"/>
-      <c r="J66" s="107"/>
-      <c r="K66" s="107"/>
-      <c r="L66" s="107"/>
-      <c r="M66" s="107"/>
-      <c r="N66" s="107"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="108" t="s">
+      <c r="C66" s="107"/>
+      <c r="D66" s="75"/>
+      <c r="E66" s="108"/>
+      <c r="F66" s="108"/>
+      <c r="G66" s="108"/>
+      <c r="H66" s="108"/>
+      <c r="I66" s="108"/>
+      <c r="J66" s="108"/>
+      <c r="K66" s="108"/>
+      <c r="L66" s="108"/>
+      <c r="M66" s="108"/>
+      <c r="N66" s="108"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B67" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="C67" s="109"/>
-      <c r="D67" s="77"/>
-      <c r="E67" s="110"/>
-      <c r="F67" s="110"/>
-      <c r="G67" s="110"/>
-      <c r="H67" s="110"/>
-      <c r="I67" s="110"/>
-      <c r="J67" s="110"/>
-      <c r="K67" s="110"/>
-      <c r="L67" s="110"/>
-      <c r="M67" s="110"/>
-      <c r="N67" s="110"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="108" t="s">
+      <c r="C67" s="110"/>
+      <c r="D67" s="78"/>
+      <c r="E67" s="111"/>
+      <c r="F67" s="111"/>
+      <c r="G67" s="111"/>
+      <c r="H67" s="111"/>
+      <c r="I67" s="111"/>
+      <c r="J67" s="111"/>
+      <c r="K67" s="111"/>
+      <c r="L67" s="111"/>
+      <c r="M67" s="111"/>
+      <c r="N67" s="111"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B69" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="C69" s="109"/>
-      <c r="D69" s="77"/>
-      <c r="E69" s="107"/>
-      <c r="F69" s="107"/>
-      <c r="G69" s="107"/>
-      <c r="H69" s="107"/>
-      <c r="I69" s="107"/>
-      <c r="J69" s="107"/>
-      <c r="K69" s="107"/>
-      <c r="L69" s="107"/>
-      <c r="M69" s="107"/>
-      <c r="N69" s="107"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="108" t="s">
+      <c r="C69" s="110"/>
+      <c r="D69" s="78"/>
+      <c r="E69" s="108"/>
+      <c r="F69" s="108"/>
+      <c r="G69" s="108"/>
+      <c r="H69" s="108"/>
+      <c r="I69" s="108"/>
+      <c r="J69" s="108"/>
+      <c r="K69" s="108"/>
+      <c r="L69" s="108"/>
+      <c r="M69" s="108"/>
+      <c r="N69" s="108"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B70" s="109" t="s">
         <v>82</v>
       </c>
-      <c r="C70" s="109"/>
-      <c r="D70" s="77"/>
-      <c r="E70" s="110"/>
-      <c r="F70" s="110"/>
-      <c r="G70" s="110"/>
-      <c r="H70" s="110"/>
-      <c r="I70" s="110"/>
-      <c r="J70" s="110"/>
-      <c r="K70" s="110"/>
-      <c r="L70" s="110"/>
-      <c r="M70" s="110"/>
-      <c r="N70" s="110"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C70" s="110"/>
+      <c r="D70" s="78"/>
+      <c r="E70" s="111"/>
+      <c r="F70" s="111"/>
+      <c r="G70" s="111"/>
+      <c r="H70" s="111"/>
+      <c r="I70" s="111"/>
+      <c r="J70" s="111"/>
+      <c r="K70" s="111"/>
+      <c r="L70" s="111"/>
+      <c r="M70" s="111"/>
+      <c r="N70" s="111"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E72" s="110"/>
+      <c r="E72" s="111"/>
     </row>
   </sheetData>
   <mergeCells count="86">
@@ -2929,279 +2924,279 @@
   <dimension ref="B2:E30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="111" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="111" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="49.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="111" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="112" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="112" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="113" width="49.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="112" width="15.71"/>
   </cols>
   <sheetData>
-    <row r="2" s="112" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="113" t="s">
+    <row r="2" s="114" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="115" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="113" t="s">
+      <c r="C2" s="115" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="113" t="s">
+      <c r="D2" s="115" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="113" t="s">
+      <c r="E2" s="115" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="114" t="n">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="116" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="115" t="n">
+      <c r="C3" s="117" t="n">
         <v>43935</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="118" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="114" t="s">
+      <c r="E3" s="116" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="117" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="119" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="118" t="n">
+      <c r="C4" s="120" t="n">
         <v>43937</v>
       </c>
-      <c r="D4" s="119" t="s">
+      <c r="D4" s="121" t="s">
         <v>90</v>
       </c>
-      <c r="E4" s="117" t="s">
+      <c r="E4" s="119" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="117" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="119" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="118" t="n">
+      <c r="C5" s="120" t="n">
         <v>43990</v>
       </c>
-      <c r="D5" s="119" t="s">
+      <c r="D5" s="121" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="117" t="s">
+      <c r="E5" s="119" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="117" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="119" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="118" t="n">
+      <c r="C6" s="120" t="n">
         <v>44127</v>
       </c>
-      <c r="D6" s="119" t="s">
+      <c r="D6" s="121" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="117" t="s">
+      <c r="E6" s="119" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="117" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="119" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="117"/>
-      <c r="D7" s="119" t="s">
+      <c r="C7" s="119"/>
+      <c r="D7" s="121" t="s">
         <v>95</v>
       </c>
-      <c r="E7" s="117" t="s">
+      <c r="E7" s="119" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="117" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="119" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="118" t="n">
+      <c r="C8" s="120" t="n">
         <v>44239</v>
       </c>
-      <c r="D8" s="119" t="s">
+      <c r="D8" s="121" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="117" t="s">
+      <c r="E8" s="119" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="117" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="119" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="118" t="n">
+      <c r="C9" s="120" t="n">
         <v>44302</v>
       </c>
-      <c r="D9" s="119" t="s">
+      <c r="D9" s="121" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="117" t="s">
+      <c r="E9" s="119" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="117" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="119" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="118" t="n">
+      <c r="C10" s="120" t="n">
         <v>44312</v>
       </c>
-      <c r="D10" s="119" t="s">
+      <c r="D10" s="121" t="s">
         <v>98</v>
       </c>
-      <c r="E10" s="117" t="s">
+      <c r="E10" s="119" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="117" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="119" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="118" t="n">
+      <c r="C11" s="120" t="n">
         <v>44566</v>
       </c>
-      <c r="D11" s="119" t="s">
+      <c r="D11" s="121" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="117" t="s">
+      <c r="E11" s="119" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="117" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="119" t="n">
         <v>10</v>
       </c>
-      <c r="C12" s="118" t="n">
+      <c r="C12" s="120" t="n">
         <v>44938</v>
       </c>
-      <c r="D12" s="119" t="s">
+      <c r="D12" s="121" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="117" t="s">
+      <c r="E12" s="119" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="117" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="119" t="n">
         <v>11</v>
       </c>
-      <c r="C13" s="118" t="n">
+      <c r="C13" s="120" t="n">
         <v>45554</v>
       </c>
-      <c r="D13" s="119" t="s">
+      <c r="D13" s="121" t="s">
         <v>101</v>
       </c>
-      <c r="E13" s="117" t="s">
+      <c r="E13" s="119" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="117"/>
-      <c r="C14" s="117"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="117"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="117"/>
-      <c r="C15" s="117"/>
-      <c r="D15" s="119"/>
-      <c r="E15" s="117"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="117"/>
-      <c r="C16" s="117"/>
-      <c r="D16" s="119"/>
-      <c r="E16" s="117"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="117"/>
-      <c r="C17" s="117"/>
-      <c r="D17" s="119"/>
-      <c r="E17" s="117"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="117"/>
-      <c r="C18" s="117"/>
-      <c r="D18" s="119"/>
-      <c r="E18" s="117"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="117"/>
-      <c r="C19" s="117"/>
-      <c r="D19" s="119"/>
-      <c r="E19" s="117"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="117"/>
-      <c r="C20" s="117"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="117"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="117"/>
-      <c r="C21" s="117"/>
-      <c r="D21" s="119"/>
-      <c r="E21" s="117"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="117"/>
-      <c r="C22" s="117"/>
-      <c r="D22" s="119"/>
-      <c r="E22" s="117"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="117"/>
-      <c r="C23" s="117"/>
-      <c r="D23" s="119"/>
-      <c r="E23" s="117"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="117"/>
-      <c r="C24" s="117"/>
-      <c r="D24" s="119"/>
-      <c r="E24" s="117"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="117"/>
-      <c r="C25" s="117"/>
-      <c r="D25" s="119"/>
-      <c r="E25" s="117"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="117"/>
-      <c r="C26" s="117"/>
-      <c r="D26" s="119"/>
-      <c r="E26" s="117"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="117"/>
-      <c r="C27" s="117"/>
-      <c r="D27" s="119"/>
-      <c r="E27" s="117"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="117"/>
-      <c r="C28" s="117"/>
-      <c r="D28" s="119"/>
-      <c r="E28" s="117"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="117"/>
-      <c r="C29" s="117"/>
-      <c r="D29" s="119"/>
-      <c r="E29" s="117"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="120"/>
-      <c r="C30" s="120"/>
-      <c r="D30" s="121"/>
-      <c r="E30" s="120"/>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="121"/>
+      <c r="E14" s="119"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="119"/>
+      <c r="C15" s="119"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="119"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="119"/>
+      <c r="C16" s="119"/>
+      <c r="D16" s="121"/>
+      <c r="E16" s="119"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="119"/>
+      <c r="C17" s="119"/>
+      <c r="D17" s="121"/>
+      <c r="E17" s="119"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="119"/>
+      <c r="C18" s="119"/>
+      <c r="D18" s="121"/>
+      <c r="E18" s="119"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="119"/>
+      <c r="C19" s="119"/>
+      <c r="D19" s="121"/>
+      <c r="E19" s="119"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="119"/>
+      <c r="C20" s="119"/>
+      <c r="D20" s="121"/>
+      <c r="E20" s="119"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="119"/>
+      <c r="C21" s="119"/>
+      <c r="D21" s="121"/>
+      <c r="E21" s="119"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="119"/>
+      <c r="C22" s="119"/>
+      <c r="D22" s="121"/>
+      <c r="E22" s="119"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="119"/>
+      <c r="C23" s="119"/>
+      <c r="D23" s="121"/>
+      <c r="E23" s="119"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="119"/>
+      <c r="C24" s="119"/>
+      <c r="D24" s="121"/>
+      <c r="E24" s="119"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="119"/>
+      <c r="C25" s="119"/>
+      <c r="D25" s="121"/>
+      <c r="E25" s="119"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="119"/>
+      <c r="C26" s="119"/>
+      <c r="D26" s="121"/>
+      <c r="E26" s="119"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="119"/>
+      <c r="C27" s="119"/>
+      <c r="D27" s="121"/>
+      <c r="E27" s="119"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="119"/>
+      <c r="C28" s="119"/>
+      <c r="D28" s="121"/>
+      <c r="E28" s="119"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="119"/>
+      <c r="C29" s="119"/>
+      <c r="D29" s="121"/>
+      <c r="E29" s="119"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="122"/>
+      <c r="C30" s="122"/>
+      <c r="D30" s="123"/>
+      <c r="E30" s="122"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Fix: receptversie werd als datum getoond, datumformaat naar dd-mm-jjjj, Changes-cel vergroot
- E67 (Recipe version, bv. '11.1') erfde de datum-opmaak van de oude
  'Date'-cel uit het originele sjabloon -- nu General, en de writer schrijft
  'm voortaan altijd geforceerd als tekst ({text: ...}) zodat een
  getal-achtige waarde nooit als datum/getal geinterpreteerd kan worden.
- E70 (Date): schrijft nu dd-mm-jjjj i.p.v. het rauwe yyyy-mm-dd uit de
  database (psFormatteerDatumDDMMJJJJ), en de cel-opmaak zelf staat ook op
  dd-mm-yyyy voor het geval er ooit een echte datumwaarde in komt.
- E72 (Changes) erfde per ongeluk ook de datum-opmaak toen die cel vorige
  sessie werd aangemaakt -- teruggezet naar tekst, nu samengevoegd tot
  E72:N72, tekstterugloop aan, rijhoogte naar 60.
</commit_message>
<xml_diff>
--- a/productsheet-generator/Product_Sheet_sjabloon.xlsx
+++ b/productsheet-generator/Product_Sheet_sjabloon.xlsx
@@ -336,13 +336,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="General"/>
     <numFmt numFmtId="168" formatCode="@"/>
     <numFmt numFmtId="169" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="170" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -746,7 +747,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="125">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1191,8 +1192,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="170" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2756,16 +2761,16 @@
       </c>
       <c r="C67" s="110"/>
       <c r="D67" s="78"/>
-      <c r="E67" s="111"/>
-      <c r="F67" s="111"/>
-      <c r="G67" s="111"/>
-      <c r="H67" s="111"/>
-      <c r="I67" s="111"/>
-      <c r="J67" s="111"/>
-      <c r="K67" s="111"/>
-      <c r="L67" s="111"/>
-      <c r="M67" s="111"/>
-      <c r="N67" s="111"/>
+      <c r="E67" s="108"/>
+      <c r="F67" s="108"/>
+      <c r="G67" s="108"/>
+      <c r="H67" s="108"/>
+      <c r="I67" s="108"/>
+      <c r="J67" s="108"/>
+      <c r="K67" s="108"/>
+      <c r="L67" s="108"/>
+      <c r="M67" s="108"/>
+      <c r="N67" s="108"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="109" t="s">
@@ -2801,14 +2806,23 @@
       <c r="M70" s="111"/>
       <c r="N70" s="111"/>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E72" s="111"/>
+      <c r="E72" s="112"/>
+      <c r="F72" s="112"/>
+      <c r="G72" s="112"/>
+      <c r="H72" s="112"/>
+      <c r="I72" s="112"/>
+      <c r="J72" s="112"/>
+      <c r="K72" s="112"/>
+      <c r="L72" s="112"/>
+      <c r="M72" s="112"/>
+      <c r="N72" s="112"/>
     </row>
   </sheetData>
-  <mergeCells count="86">
+  <mergeCells count="87">
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="E4:N4"/>
@@ -2895,6 +2909,7 @@
     <mergeCell ref="E67:N67"/>
     <mergeCell ref="E69:N69"/>
     <mergeCell ref="E70:N70"/>
+    <mergeCell ref="E72:N72"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Q16" r:id="rId1" display="mailto:daniel.schappert@jopenbier.nl"/>
@@ -2924,279 +2939,279 @@
   <dimension ref="B2:E30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="112" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="112" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="113" width="49.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="112" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="113" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="113" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="114" width="49.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="113" width="15.71"/>
   </cols>
   <sheetData>
-    <row r="2" s="114" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="115" t="s">
+    <row r="2" s="115" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="116" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="115" t="s">
+      <c r="C2" s="116" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="115" t="s">
+      <c r="D2" s="116" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="115" t="s">
+      <c r="E2" s="116" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="116" t="n">
+      <c r="B3" s="117" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="117" t="n">
+      <c r="C3" s="118" t="n">
         <v>43935</v>
       </c>
-      <c r="D3" s="118" t="s">
+      <c r="D3" s="119" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="116" t="s">
+      <c r="E3" s="117" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="119" t="n">
+      <c r="B4" s="120" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="120" t="n">
+      <c r="C4" s="121" t="n">
         <v>43937</v>
       </c>
-      <c r="D4" s="121" t="s">
+      <c r="D4" s="122" t="s">
         <v>90</v>
       </c>
-      <c r="E4" s="119" t="s">
+      <c r="E4" s="120" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="119" t="n">
+      <c r="B5" s="120" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="120" t="n">
+      <c r="C5" s="121" t="n">
         <v>43990</v>
       </c>
-      <c r="D5" s="121" t="s">
+      <c r="D5" s="122" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="119" t="s">
+      <c r="E5" s="120" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="119" t="n">
+      <c r="B6" s="120" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="120" t="n">
+      <c r="C6" s="121" t="n">
         <v>44127</v>
       </c>
-      <c r="D6" s="121" t="s">
+      <c r="D6" s="122" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="119" t="s">
+      <c r="E6" s="120" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="119" t="n">
+      <c r="B7" s="120" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="119"/>
-      <c r="D7" s="121" t="s">
+      <c r="C7" s="120"/>
+      <c r="D7" s="122" t="s">
         <v>95</v>
       </c>
-      <c r="E7" s="119" t="s">
+      <c r="E7" s="120" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="119" t="n">
+      <c r="B8" s="120" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="120" t="n">
+      <c r="C8" s="121" t="n">
         <v>44239</v>
       </c>
-      <c r="D8" s="121" t="s">
+      <c r="D8" s="122" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="119" t="s">
+      <c r="E8" s="120" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="119" t="n">
+      <c r="B9" s="120" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="120" t="n">
+      <c r="C9" s="121" t="n">
         <v>44302</v>
       </c>
-      <c r="D9" s="121" t="s">
+      <c r="D9" s="122" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="119" t="s">
+      <c r="E9" s="120" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="119" t="n">
+      <c r="B10" s="120" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="120" t="n">
+      <c r="C10" s="121" t="n">
         <v>44312</v>
       </c>
-      <c r="D10" s="121" t="s">
+      <c r="D10" s="122" t="s">
         <v>98</v>
       </c>
-      <c r="E10" s="119" t="s">
+      <c r="E10" s="120" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="119" t="n">
+      <c r="B11" s="120" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="120" t="n">
+      <c r="C11" s="121" t="n">
         <v>44566</v>
       </c>
-      <c r="D11" s="121" t="s">
+      <c r="D11" s="122" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="119" t="s">
+      <c r="E11" s="120" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="119" t="n">
+      <c r="B12" s="120" t="n">
         <v>10</v>
       </c>
-      <c r="C12" s="120" t="n">
+      <c r="C12" s="121" t="n">
         <v>44938</v>
       </c>
-      <c r="D12" s="121" t="s">
+      <c r="D12" s="122" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="119" t="s">
+      <c r="E12" s="120" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="119" t="n">
+      <c r="B13" s="120" t="n">
         <v>11</v>
       </c>
-      <c r="C13" s="120" t="n">
+      <c r="C13" s="121" t="n">
         <v>45554</v>
       </c>
-      <c r="D13" s="121" t="s">
+      <c r="D13" s="122" t="s">
         <v>101</v>
       </c>
-      <c r="E13" s="119" t="s">
+      <c r="E13" s="120" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="121"/>
-      <c r="E14" s="119"/>
+      <c r="B14" s="120"/>
+      <c r="C14" s="120"/>
+      <c r="D14" s="122"/>
+      <c r="E14" s="120"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="119"/>
-      <c r="C15" s="119"/>
-      <c r="D15" s="121"/>
-      <c r="E15" s="119"/>
+      <c r="B15" s="120"/>
+      <c r="C15" s="120"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="120"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="119"/>
-      <c r="C16" s="119"/>
-      <c r="D16" s="121"/>
-      <c r="E16" s="119"/>
+      <c r="B16" s="120"/>
+      <c r="C16" s="120"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="120"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="119"/>
-      <c r="C17" s="119"/>
-      <c r="D17" s="121"/>
-      <c r="E17" s="119"/>
+      <c r="B17" s="120"/>
+      <c r="C17" s="120"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="120"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="119"/>
-      <c r="C18" s="119"/>
-      <c r="D18" s="121"/>
-      <c r="E18" s="119"/>
+      <c r="B18" s="120"/>
+      <c r="C18" s="120"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="120"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="119"/>
-      <c r="C19" s="119"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="119"/>
+      <c r="B19" s="120"/>
+      <c r="C19" s="120"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="120"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="121"/>
-      <c r="E20" s="119"/>
+      <c r="B20" s="120"/>
+      <c r="C20" s="120"/>
+      <c r="D20" s="122"/>
+      <c r="E20" s="120"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="119"/>
-      <c r="C21" s="119"/>
-      <c r="D21" s="121"/>
-      <c r="E21" s="119"/>
+      <c r="B21" s="120"/>
+      <c r="C21" s="120"/>
+      <c r="D21" s="122"/>
+      <c r="E21" s="120"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="119"/>
-      <c r="C22" s="119"/>
-      <c r="D22" s="121"/>
-      <c r="E22" s="119"/>
+      <c r="B22" s="120"/>
+      <c r="C22" s="120"/>
+      <c r="D22" s="122"/>
+      <c r="E22" s="120"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="119"/>
-      <c r="C23" s="119"/>
-      <c r="D23" s="121"/>
-      <c r="E23" s="119"/>
+      <c r="B23" s="120"/>
+      <c r="C23" s="120"/>
+      <c r="D23" s="122"/>
+      <c r="E23" s="120"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="119"/>
-      <c r="C24" s="119"/>
-      <c r="D24" s="121"/>
-      <c r="E24" s="119"/>
+      <c r="B24" s="120"/>
+      <c r="C24" s="120"/>
+      <c r="D24" s="122"/>
+      <c r="E24" s="120"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="119"/>
-      <c r="C25" s="119"/>
-      <c r="D25" s="121"/>
-      <c r="E25" s="119"/>
+      <c r="B25" s="120"/>
+      <c r="C25" s="120"/>
+      <c r="D25" s="122"/>
+      <c r="E25" s="120"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="119"/>
-      <c r="C26" s="119"/>
-      <c r="D26" s="121"/>
-      <c r="E26" s="119"/>
+      <c r="B26" s="120"/>
+      <c r="C26" s="120"/>
+      <c r="D26" s="122"/>
+      <c r="E26" s="120"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="119"/>
-      <c r="C27" s="119"/>
-      <c r="D27" s="121"/>
-      <c r="E27" s="119"/>
+      <c r="B27" s="120"/>
+      <c r="C27" s="120"/>
+      <c r="D27" s="122"/>
+      <c r="E27" s="120"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="119"/>
-      <c r="C28" s="119"/>
-      <c r="D28" s="121"/>
-      <c r="E28" s="119"/>
+      <c r="B28" s="120"/>
+      <c r="C28" s="120"/>
+      <c r="D28" s="122"/>
+      <c r="E28" s="120"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="119"/>
-      <c r="C29" s="119"/>
-      <c r="D29" s="121"/>
-      <c r="E29" s="119"/>
+      <c r="B29" s="120"/>
+      <c r="C29" s="120"/>
+      <c r="D29" s="122"/>
+      <c r="E29" s="120"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="122"/>
-      <c r="C30" s="122"/>
-      <c r="D30" s="123"/>
-      <c r="E30" s="122"/>
+      <c r="B30" s="123"/>
+      <c r="C30" s="123"/>
+      <c r="D30" s="124"/>
+      <c r="E30" s="123"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Restjes uit het originele sjabloon volledig verwijderd (mailto-lijst, allergenen-toelichting, proefleestip)
Deze stonden nog in kolom P/Q (rijen 16-23 en 42-47) -- bleken bij de eerdere
opschoning niet daadwerkelijk gewist te zijn ondanks dat die stap toen wel
leek te slagen voor de andere cellen. Nu stuk voor stuk gecontroleerd en
verwijderd; geen losse hyperlink-relaties achtergebleven.
</commit_message>
<xml_diff>
--- a/productsheet-generator/Product_Sheet_sjabloon.xlsx
+++ b/productsheet-generator/Product_Sheet_sjabloon.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="89">
   <si>
     <t xml:space="preserve">PRODUCT SHEET</t>
   </si>
@@ -68,15 +68,9 @@
     <t xml:space="preserve"> - Yeast</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:daniel.schappert@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Eindproduct specificatie</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:laboratorium@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Parameter</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
     <t xml:space="preserve">Spec.</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:michel.ordeman@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Origineel extract</t>
   </si>
   <si>
@@ -107,9 +98,6 @@
     <t xml:space="preserve">&lt;</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:roel.vanderstaak@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rest extract</t>
   </si>
   <si>
@@ -119,9 +107,6 @@
     <t xml:space="preserve">g/l</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:bas.weijers@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alcohol</t>
   </si>
   <si>
@@ -131,9 +116,6 @@
     <t xml:space="preserve">CO2 cans</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:eric.vanderlugt@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bitterness</t>
   </si>
   <si>
@@ -146,18 +128,12 @@
     <t xml:space="preserve">ppb</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:Berend.otten@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Color</t>
   </si>
   <si>
     <t xml:space="preserve">Headspace O2</t>
   </si>
   <si>
-    <t xml:space="preserve">mailto:michelle.vanderklauw@jopenbier.nl</t>
-  </si>
-  <si>
     <t xml:space="preserve">pH</t>
   </si>
   <si>
@@ -200,28 +176,10 @@
     <t xml:space="preserve">Recommended drinking temperature (°C)</t>
   </si>
   <si>
-    <t xml:space="preserve">• European legislation has named 14 substances as allergens, namely: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Gluten (wheat, rye, barley, oats, spelt, khoran wheat), shellfish, egg, fish, </t>
-  </si>
-  <si>
     <t xml:space="preserve">Flavor description (words under logo, e.g., “Soft &amp; Tropica”)</t>
   </si>
   <si>
-    <t xml:space="preserve">   peanut, soy, milk (including lactose), tree nuts (8 types), celery, mustard, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  sesame, sulfite, lupin and mollusks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Tip: Have someone else proofread the product sheet. Errors that </t>
-  </si>
-  <si>
     <t xml:space="preserve">Barrel aged bier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   sneak in here can end up on the labels!</t>
   </si>
   <si>
     <t xml:space="preserve">Amount barrel aged HL</t>
@@ -1068,7 +1026,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1793,14 +1751,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P16" s="7"/>
-      <c r="Q16" s="34" t="s">
-        <v>15</v>
-      </c>
+      <c r="Q16" s="34"/>
       <c r="X16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -1815,210 +1771,196 @@
       <c r="M17" s="17"/>
       <c r="N17" s="17"/>
       <c r="P17" s="7"/>
-      <c r="Q17" s="34" t="s">
-        <v>17</v>
-      </c>
+      <c r="Q17" s="34"/>
       <c r="X17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="35" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C18" s="35"/>
       <c r="D18" s="35"/>
       <c r="E18" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="37" t="s">
-        <v>21</v>
-      </c>
       <c r="H18" s="35" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I18" s="35"/>
       <c r="J18" s="35"/>
       <c r="K18" s="35"/>
       <c r="L18" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="N18" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="N18" s="36" t="s">
-        <v>21</v>
-      </c>
       <c r="P18" s="38"/>
-      <c r="Q18" s="34" t="s">
-        <v>22</v>
-      </c>
+      <c r="Q18" s="34"/>
       <c r="X18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="39" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C19" s="39"/>
       <c r="D19" s="39"/>
       <c r="E19" s="40" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F19" s="41" t="n">
         <v>0.2</v>
       </c>
       <c r="G19" s="42"/>
       <c r="H19" s="39" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I19" s="39"/>
       <c r="J19" s="39"/>
       <c r="K19" s="39"/>
       <c r="L19" s="40" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="M19" s="43" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N19" s="44"/>
       <c r="P19" s="7"/>
-      <c r="Q19" s="34" t="s">
-        <v>28</v>
-      </c>
+      <c r="Q19" s="34"/>
       <c r="X19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="45" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="45"/>
       <c r="E20" s="46" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F20" s="41" t="n">
         <v>0.3</v>
       </c>
       <c r="G20" s="47"/>
       <c r="H20" s="45" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I20" s="45"/>
       <c r="J20" s="45"/>
       <c r="K20" s="45"/>
       <c r="L20" s="46" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="M20" s="41" t="n">
         <v>0.1</v>
       </c>
       <c r="N20" s="47"/>
       <c r="P20" s="7"/>
-      <c r="Q20" s="34" t="s">
-        <v>32</v>
-      </c>
+      <c r="Q20" s="34"/>
       <c r="X20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="45" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="45"/>
       <c r="E21" s="46" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F21" s="41" t="n">
         <v>0.5</v>
       </c>
       <c r="G21" s="47"/>
       <c r="H21" s="45" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I21" s="45"/>
       <c r="J21" s="45"/>
       <c r="K21" s="45"/>
       <c r="L21" s="46" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="M21" s="41" t="n">
         <v>0.1</v>
       </c>
       <c r="N21" s="47"/>
       <c r="P21" s="7"/>
-      <c r="Q21" s="34" t="s">
-        <v>36</v>
-      </c>
+      <c r="Q21" s="34"/>
       <c r="X21" s="8"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="45" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="45"/>
       <c r="E22" s="46" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F22" s="43" t="n">
         <v>3</v>
       </c>
       <c r="G22" s="48"/>
       <c r="H22" s="45" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I22" s="45"/>
       <c r="J22" s="45"/>
       <c r="K22" s="45"/>
       <c r="L22" s="46" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="M22" s="41" t="n">
         <v>0.1</v>
       </c>
       <c r="N22" s="48"/>
       <c r="P22" s="7"/>
-      <c r="Q22" s="34" t="s">
-        <v>41</v>
-      </c>
+      <c r="Q22" s="34"/>
       <c r="X22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="45" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="45"/>
       <c r="E23" s="46" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F23" s="43" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="48"/>
       <c r="H23" s="45" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I23" s="45"/>
       <c r="J23" s="45"/>
       <c r="K23" s="45"/>
       <c r="L23" s="46" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="M23" s="41" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N23" s="48"/>
       <c r="P23" s="7"/>
-      <c r="Q23" s="34" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q23" s="34"/>
       <c r="X23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="45" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="45"/>
@@ -2028,16 +1970,16 @@
       </c>
       <c r="G24" s="47"/>
       <c r="H24" s="49" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="I24" s="49"/>
       <c r="J24" s="49"/>
       <c r="K24" s="49"/>
       <c r="L24" s="46" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="M24" s="41" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N24" s="50" t="n">
         <v>50</v>
@@ -2047,15 +1989,15 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="51" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C25" s="52"/>
       <c r="D25" s="53"/>
       <c r="E25" s="54" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F25" s="55" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G25" s="56"/>
       <c r="H25" s="52"/>
@@ -2074,7 +2016,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="18" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C27" s="18"/>
       <c r="D27" s="23"/>
@@ -2165,7 +2107,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="17" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
@@ -2184,7 +2126,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="22" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C34" s="22"/>
       <c r="D34" s="60"/>
@@ -2208,7 +2150,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="26" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C35" s="26"/>
       <c r="D35" s="27"/>
@@ -2232,7 +2174,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="26" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C36" s="26"/>
       <c r="D36" s="27"/>
@@ -2256,7 +2198,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="26" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C37" s="26"/>
       <c r="D37" s="27"/>
@@ -2275,7 +2217,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="26" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C38" s="26"/>
       <c r="D38" s="27"/>
@@ -2294,7 +2236,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="26" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C39" s="26"/>
       <c r="D39" s="27"/>
@@ -2318,7 +2260,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="26" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C40" s="26"/>
       <c r="D40" s="27"/>
@@ -2339,7 +2281,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="26" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C41" s="26"/>
       <c r="D41" s="27"/>
@@ -2358,7 +2300,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="68" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C42" s="68"/>
       <c r="D42" s="69"/>
@@ -2372,9 +2314,7 @@
       <c r="L42" s="70"/>
       <c r="M42" s="70"/>
       <c r="N42" s="70"/>
-      <c r="P42" s="71" t="s">
-        <v>59</v>
-      </c>
+      <c r="P42" s="71"/>
       <c r="Q42" s="72"/>
       <c r="R42" s="72"/>
       <c r="S42" s="72"/>
@@ -2385,9 +2325,7 @@
       <c r="X42" s="73"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="P43" s="71" t="s">
-        <v>60</v>
-      </c>
+      <c r="P43" s="71"/>
       <c r="Q43" s="72"/>
       <c r="R43" s="72"/>
       <c r="S43" s="72"/>
@@ -2399,7 +2337,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="74" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C44" s="74"/>
       <c r="D44" s="75"/>
@@ -2413,9 +2351,7 @@
       <c r="L44" s="77"/>
       <c r="M44" s="76"/>
       <c r="N44" s="76"/>
-      <c r="P44" s="71" t="s">
-        <v>62</v>
-      </c>
+      <c r="P44" s="71"/>
       <c r="Q44" s="72"/>
       <c r="R44" s="72"/>
       <c r="S44" s="72"/>
@@ -2439,9 +2375,7 @@
       <c r="L45" s="76"/>
       <c r="M45" s="77"/>
       <c r="N45" s="77"/>
-      <c r="P45" s="71" t="s">
-        <v>63</v>
-      </c>
+      <c r="P45" s="71"/>
       <c r="Q45" s="72"/>
       <c r="R45" s="72"/>
       <c r="S45" s="72"/>
@@ -2452,14 +2386,12 @@
       <c r="X45" s="73"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="P46" s="7" t="s">
-        <v>64</v>
-      </c>
+      <c r="P46" s="7"/>
       <c r="X46" s="8"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="17" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -2473,9 +2405,7 @@
       <c r="L47" s="17"/>
       <c r="M47" s="17"/>
       <c r="N47" s="17"/>
-      <c r="P47" s="80" t="s">
-        <v>66</v>
-      </c>
+      <c r="P47" s="80"/>
       <c r="Q47" s="81"/>
       <c r="R47" s="81"/>
       <c r="S47" s="81"/>
@@ -2487,12 +2417,12 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="26" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="C48" s="26"/>
       <c r="D48" s="27"/>
       <c r="E48" s="66" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="F48" s="66"/>
       <c r="G48" s="66"/>
@@ -2506,12 +2436,12 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="26" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="C49" s="26"/>
       <c r="D49" s="27"/>
       <c r="E49" s="66" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="F49" s="66"/>
       <c r="G49" s="66"/>
@@ -2525,12 +2455,12 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="83" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="C50" s="84"/>
       <c r="D50" s="69"/>
       <c r="E50" s="85" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="F50" s="85"/>
       <c r="G50" s="85"/>
@@ -2544,7 +2474,7 @@
     </row>
     <row r="52" customFormat="false" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="86" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="C52" s="87"/>
       <c r="D52" s="23"/>
@@ -2621,7 +2551,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="17" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="17"/>
@@ -2638,7 +2568,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="26" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C59" s="26"/>
       <c r="D59" s="27"/>
@@ -2655,7 +2585,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="26" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="C60" s="26"/>
       <c r="D60" s="27"/>
@@ -2672,7 +2602,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="101" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C61" s="102"/>
       <c r="D61" s="103"/>
@@ -2689,7 +2619,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="101" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="C62" s="102"/>
       <c r="D62" s="103"/>
@@ -2706,7 +2636,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="101" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="C63" s="102"/>
       <c r="D63" s="103"/>
@@ -2723,7 +2653,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="83" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="C64" s="84"/>
       <c r="D64" s="69"/>
@@ -2740,7 +2670,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="106" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C66" s="107"/>
       <c r="D66" s="75"/>
@@ -2757,7 +2687,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="109" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="C67" s="110"/>
       <c r="D67" s="78"/>
@@ -2774,7 +2704,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="109" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="C69" s="110"/>
       <c r="D69" s="78"/>
@@ -2791,7 +2721,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="109" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="C70" s="110"/>
       <c r="D70" s="78"/>
@@ -2808,7 +2738,7 @@
     </row>
     <row r="72" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="109" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E72" s="112"/>
       <c r="F72" s="112"/>
@@ -2911,16 +2841,6 @@
     <mergeCell ref="E70:N70"/>
     <mergeCell ref="E72:N72"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="Q16" r:id="rId1" display="mailto:daniel.schappert@jopenbier.nl"/>
-    <hyperlink ref="Q17" r:id="rId2" display="mailto:laboratorium@jopenbier.nl"/>
-    <hyperlink ref="Q18" r:id="rId3" display="mailto:michel.ordeman@jopenbier.nl"/>
-    <hyperlink ref="Q19" r:id="rId4" display="mailto:roel.vanderstaak@jopenbier.nl"/>
-    <hyperlink ref="Q20" r:id="rId5" display="mailto:bas.weijers@jopenbier.nl"/>
-    <hyperlink ref="Q21" r:id="rId6" display="mailto:eric.vanderlugt@jopenbier.nl"/>
-    <hyperlink ref="Q22" r:id="rId7" display="mailto:Berend.otten@jopenbier.nl"/>
-    <hyperlink ref="Q23" r:id="rId8" display="mailto:michelle.vanderklauw@jopenbier.nl"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2947,16 +2867,16 @@
   <sheetData>
     <row r="2" s="115" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="116" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="C2" s="116" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="D2" s="116" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="E2" s="116" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2967,10 +2887,10 @@
         <v>43935</v>
       </c>
       <c r="D3" s="119" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="E3" s="117" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2981,10 +2901,10 @@
         <v>43937</v>
       </c>
       <c r="D4" s="122" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="E4" s="120" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2995,10 +2915,10 @@
         <v>43990</v>
       </c>
       <c r="D5" s="122" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E5" s="120" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3009,10 +2929,10 @@
         <v>44127</v>
       </c>
       <c r="D6" s="122" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E6" s="120" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3021,10 +2941,10 @@
       </c>
       <c r="C7" s="120"/>
       <c r="D7" s="122" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="E7" s="120" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3035,10 +2955,10 @@
         <v>44239</v>
       </c>
       <c r="D8" s="122" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E8" s="120" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3049,10 +2969,10 @@
         <v>44302</v>
       </c>
       <c r="D9" s="122" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="E9" s="120" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3063,10 +2983,10 @@
         <v>44312</v>
       </c>
       <c r="D10" s="122" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="E10" s="120" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3077,10 +2997,10 @@
         <v>44566</v>
       </c>
       <c r="D11" s="122" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="E11" s="120" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3091,10 +3011,10 @@
         <v>44938</v>
       </c>
       <c r="D12" s="122" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E12" s="120" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3105,10 +3025,10 @@
         <v>45554</v>
       </c>
       <c r="D13" s="122" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="E13" s="120" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>